<commit_message>
feat: add process documentation and organize datasets for Malos Manejos analysis
</commit_message>
<xml_diff>
--- a/Agentes/Agente_Malos_Manejos/Ejemplo/Malos Manejos Procesados/Malos manejos 1-13 julio Mismatches.xlsx
+++ b/Agentes/Agente_Malos_Manejos/Ejemplo/Malos Manejos Procesados/Malos manejos 1-13 julio Mismatches.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF35"/>
+  <dimension ref="A1:AF23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -585,19 +585,19 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>923D9BE7-53A6-4834-A88B-EA3D7B142908</t>
+          <t>6686EB1E-3B2A-4317-9420-10DBCFF06F61</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10D11A27-34C7-46C5-83F0-73252776BD71</t>
+          <t>461CF3A4-6E6A-4A85-9A89-DFB9756B36D7</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7929</v>
+        <v>9326</v>
       </c>
       <c r="D2" t="n">
-        <v>5129</v>
+        <v>7156</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -606,17 +606,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>BOG Y SABANA</t>
+          <t>CARIBE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>CUNDINAMARCA</t>
+          <t>CESAR</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>BOGOTÁ, D.C.</t>
+          <t>VALLEDUPAR</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -647,17 +647,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>3273 5625 5760 C HALL TRINIDAD GALAN GAM - 7929</t>
+          <t>7156 C EXITO CENTRO VALLEDUPAR - 9326 - TBS - DIEBOLD</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>SGIII-7929-9-2</t>
+          <t>SGIII-9326-2-1</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGNETICO HALL ENTRADA PRINCIPAL CAJEROS </t>
+          <t>MICROSUICHE TAPA TECLADO CAJERO</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -670,22 +670,18 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>kelly aguirre</t>
+          <t>Laura Valentina Restrepo Jaramillo</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
+          <t>Falso positivo</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr">
         <is>
-          <t>FUNCIONARIOS</t>
+          <t>TRANSBANK</t>
         </is>
       </c>
       <c r="X2">
@@ -702,43 +698,43 @@
         </is>
       </c>
       <c r="AB2" s="1" t="n">
-        <v>46204.11940972223</v>
+        <v>46204.29431712963</v>
       </c>
       <c r="AC2" s="1" t="n">
-        <v>46204.11946759259</v>
+        <v>46204.294375</v>
       </c>
       <c r="AD2" s="1" t="n">
-        <v>46204.1303125</v>
+        <v>46204.36144675926</v>
       </c>
       <c r="AE2" t="n">
-        <v>942</v>
+        <v>5800</v>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>[2026-07-01 02:52:06] kelly aguirre: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ || [2026-07-01 02:52:07] kelly aguirre: [SOP:3] Documentando ✅ || [2026-07-01 02:52:56] kelly aguirre: Por video se observa al momento de la     activación que en el punto esta TDV AT || [2026-07-01 02:53:09] kelly aguirre: PERSONAL DE LA TDV EN SITIO NO REALIZA BYPASS DE LA ZONA EN ACTIVACION LA CUAL OCASIONA ACTIVACIONES</t>
+          <t>[2026-07-01 07:03:59] Laura Valentina Restrepo Jaramillo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-01 07:04:40] Laura Valentina Restrepo Jaramillo: Se verifica por video cámara relacionada en tiempo real, TDV en el punto en aparente normalidad bk || [2026-07-01 07:04:46] Laura Valentina Restrepo Jaramillo: Activación generada por desarme inoportuno</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>923D9BE7-53A6-4834-A88B-EA3D7B142908</t>
+          <t>BF2D210F-FC82-425B-8A8B-5CB6EC3192D7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>A4E71697-77A0-4C3A-8D78-6D4A2897916B</t>
+          <t>D0783D27-CA4F-4974-AE08-0F696349FBF4</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7929</v>
+        <v>1666</v>
       </c>
       <c r="D3" t="n">
-        <v>5129</v>
+        <v>666</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>ATM</t>
+          <t>Sucursal</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -757,7 +753,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -769,37 +765,37 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
+          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>activación perimetral</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>activación perimetral atm</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>3273 5625 5760 C HALL TRINIDAD GALAN GAM - 7929</t>
+          <t>0666 S PARK WAY - 1666</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>SGIII-7929-10-2</t>
+          <t>Honeywell7810PC-1666-8-1</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>INFRARROJO HALL CAJEROS</t>
+          <t xml:space="preserve">TAMPER CAJA MARNELL </t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>SGIII</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="S3" t="n">
@@ -807,19 +803,15 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>kelly aguirre</t>
+          <t>Adier Cuitiva Mayo</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
+          <t>Falso positivo</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr">
         <is>
           <t>FUNCIONARIOS</t>
@@ -831,7 +823,7 @@
       </c>
       <c r="Y3" t="inlineStr"/>
       <c r="Z3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
@@ -839,39 +831,43 @@
         </is>
       </c>
       <c r="AB3" s="1" t="n">
-        <v>46204.11942129629</v>
+        <v>46204.37851851852</v>
       </c>
       <c r="AC3" s="1" t="n">
-        <v>46204.11951388889</v>
+        <v>46204.37858796296</v>
       </c>
       <c r="AD3" s="1" t="n">
-        <v>46204.1303125</v>
+        <v>46204.56600694444</v>
       </c>
       <c r="AE3" t="n">
-        <v>941</v>
-      </c>
-      <c r="AF3" t="inlineStr"/>
+        <v>16199</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>[2026-07-01 09:05:17] Adier Cuitiva Mayo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-01 09:05:57] Adier Cuitiva Mayo: Se verifica por video cámara relacionada en tiempo real, en el punto en aparente normalidad || [2026-07-01 09:06:07] Adier Cuitiva Mayo: En desmunte obras</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A1197B15-A11C-4306-BFA8-2CE8F60E06AA</t>
+          <t>BF2D210F-FC82-425B-8A8B-5CB6EC3192D7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0E3BC721-D556-406A-9EE7-BDC720908803</t>
+          <t>79046292-2CFD-4C5C-9545-F9DCA73E42A8</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7929</v>
+        <v>1666</v>
       </c>
       <c r="D4" t="n">
-        <v>5129</v>
+        <v>666</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ATM</t>
+          <t>Sucursal</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -890,7 +886,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -902,37 +898,37 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
+          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>activación perimetral</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>activación perimetral atm</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>3273 5625 5760 C HALL TRINIDAD GALAN GAM - 7929</t>
+          <t>0666 S PARK WAY - 1666</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>SGIII-7929-10-2</t>
+          <t>Honeywell7810PC-1666-84-1</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>INFRARROJO HALL CAJEROS</t>
+          <t xml:space="preserve">TAMPER CENTRAL PARK WAY </t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>SGIII</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="S4" t="n">
@@ -940,19 +936,15 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>Neidy Martínez</t>
+          <t>Adier Cuitiva Mayo</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
+          <t>Falso positivo</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr">
         <is>
           <t>FUNCIONARIOS</t>
@@ -964,7 +956,7 @@
       </c>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
@@ -972,39 +964,35 @@
         </is>
       </c>
       <c r="AB4" s="1" t="n">
-        <v>46204.13042824074</v>
+        <v>46204.37854166667</v>
       </c>
       <c r="AC4" s="1" t="n">
-        <v>46204.13048611111</v>
+        <v>46204.37858796296</v>
       </c>
       <c r="AD4" s="1" t="n">
-        <v>46204.13655092593</v>
+        <v>46204.56600694444</v>
       </c>
       <c r="AE4" t="n">
-        <v>529</v>
-      </c>
-      <c r="AF4" t="inlineStr">
-        <is>
-          <t>[2026-07-01 03:09:04] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-01 03:10:02] Neidy Martínez: Se valida por video command se observa tdv ATLAS en el sitio     Mal manejo, personal en sitio no realiza bypass de la zona 24 Horas</t>
-        </is>
-      </c>
+        <v>16197</v>
+      </c>
+      <c r="AF4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6686EB1E-3B2A-4317-9420-10DBCFF06F61</t>
+          <t>0CF7D86D-118E-4E73-813B-DA90EB515E49</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>461CF3A4-6E6A-4A85-9A89-DFB9756B36D7</t>
+          <t>8D6AA44A-CE22-48B1-8CED-5CBB40FBEE16</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9326</v>
+        <v>6997</v>
       </c>
       <c r="D5" t="n">
-        <v>7156</v>
+        <v>8726</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1013,17 +1001,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>CARIBE</t>
+          <t>SUR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CESAR</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>VALLEDUPAR</t>
+          <t>CALI</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -1054,22 +1042,22 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>7156 C EXITO CENTRO VALLEDUPAR - 9326 - TBS - DIEBOLD</t>
+          <t>8726 8727 8728 8729 C MF HALL CALI PRINCIPAL - 6997 - AdminSUC - DIEBOLD</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>SGIII-9326-2-1</t>
+          <t>Honeywell7810PC-6997-16-1</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>MICROSUICHE TAPA TECLADO CAJERO</t>
+          <t xml:space="preserve">MAGNETICO PUERTA PASILLO CUARTO TECNICO CAJERO </t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>SGIII</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="S5" t="n">
@@ -1077,7 +1065,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>Laura Valentina Restrepo Jaramillo</t>
+          <t>JUAN RODOLFO VASQUEZ ALZATE</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1088,7 +1076,7 @@
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
-          <t>TRANSBANK</t>
+          <t>FUNCIONARIOS</t>
         </is>
       </c>
       <c r="X5">
@@ -1097,7 +1085,7 @@
       </c>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
@@ -1105,62 +1093,62 @@
         </is>
       </c>
       <c r="AB5" s="1" t="n">
-        <v>46204.29431712963</v>
+        <v>46205.00329861111</v>
       </c>
       <c r="AC5" s="1" t="n">
-        <v>46204.294375</v>
+        <v>46205.00336805556</v>
       </c>
       <c r="AD5" s="1" t="n">
-        <v>46204.36144675926</v>
+        <v>46205.06435185186</v>
       </c>
       <c r="AE5" t="n">
-        <v>5800</v>
+        <v>5275</v>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>[2026-07-01 07:03:59] Laura Valentina Restrepo Jaramillo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-01 07:04:40] Laura Valentina Restrepo Jaramillo: Se verifica por video cámara relacionada en tiempo real, TDV en el punto en aparente normalidad bk || [2026-07-01 07:04:46] Laura Valentina Restrepo Jaramillo: Activación generada por desarme inoportuno</t>
+          <t>[2026-07-02 00:07:16] JUAN RODOLFO VASQUEZ ALZATE: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 00:07:24] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BF2D210F-FC82-425B-8A8B-5CB6EC3192D7</t>
+          <t>0CF7D86D-118E-4E73-813B-DA90EB515E49</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>D0783D27-CA4F-4974-AE08-0F696349FBF4</t>
+          <t>0825C3AE-74CB-4CC0-867C-0E7C79C7FDE0</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1666</v>
+        <v>6997</v>
       </c>
       <c r="D6" t="n">
-        <v>666</v>
+        <v>8726</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sucursal</t>
+          <t>ATM</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>BOG Y SABANA</t>
+          <t>SUR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CUNDINAMARCA</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>BOGOTÁ, D.C.</t>
+          <t>CALI</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
@@ -1172,32 +1160,32 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
+          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral atm</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0666 S PARK WAY - 1666</t>
+          <t>8726 8727 8728 8729 C MF HALL CALI PRINCIPAL - 6997 - AdminSUC - DIEBOLD</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-1666-8-1</t>
+          <t>Honeywell7810PC-6997-2-1</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMPER CAJA MARNELL </t>
+          <t>INFRARROJO ENTRADA HALL CAJERO</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1210,7 +1198,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>Adier Cuitiva Mayo</t>
+          <t>JUAN RODOLFO VASQUEZ ALZATE</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1230,7 +1218,7 @@
       </c>
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA6" t="inlineStr">
         <is>
@@ -1238,58 +1226,58 @@
         </is>
       </c>
       <c r="AB6" s="1" t="n">
-        <v>46204.37851851852</v>
+        <v>46205.00351851852</v>
       </c>
       <c r="AC6" s="1" t="n">
-        <v>46204.37858796296</v>
+        <v>46205.00357638889</v>
       </c>
       <c r="AD6" s="1" t="n">
-        <v>46204.56600694444</v>
+        <v>46205.06435185186</v>
       </c>
       <c r="AE6" t="n">
-        <v>16199</v>
+        <v>5256</v>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>[2026-07-01 09:05:17] Adier Cuitiva Mayo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-01 09:05:57] Adier Cuitiva Mayo: Se verifica por video cámara relacionada en tiempo real, en el punto en aparente normalidad || [2026-07-01 09:06:07] Adier Cuitiva Mayo: En desmunte obras</t>
+          <t>[2026-07-02 00:05:34] JUAN RODOLFO VASQUEZ ALZATE: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 00:05:38] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVAN FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BF2D210F-FC82-425B-8A8B-5CB6EC3192D7</t>
+          <t>0CF7D86D-118E-4E73-813B-DA90EB515E49</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>79046292-2CFD-4C5C-9545-F9DCA73E42A8</t>
+          <t>9215F0DF-62AC-435C-8599-4FC8964BC185</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1666</v>
+        <v>6997</v>
       </c>
       <c r="D7" t="n">
-        <v>666</v>
+        <v>8726</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sucursal</t>
+          <t>ATM</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>BOG Y SABANA</t>
+          <t>SUR</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>CUNDINAMARCA</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>BOGOTÁ, D.C.</t>
+          <t>CALI</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -1305,32 +1293,32 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
+          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral atm</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0666 S PARK WAY - 1666</t>
+          <t>8726 8727 8728 8729 C MF HALL CALI PRINCIPAL - 6997 - AdminSUC - DIEBOLD</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-1666-84-1</t>
+          <t>Honeywell7810PC-6997-12-1</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMPER CENTRAL PARK WAY </t>
+          <t>INFRARROJO PASILLO ATRAS CAJERO</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -1343,7 +1331,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>Adier Cuitiva Mayo</t>
+          <t>JUAN RODOLFO VASQUEZ ALZATE</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1363,7 +1351,7 @@
       </c>
       <c r="Y7" t="inlineStr"/>
       <c r="Z7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -1371,18 +1359,22 @@
         </is>
       </c>
       <c r="AB7" s="1" t="n">
-        <v>46204.37854166667</v>
+        <v>46205.00357638889</v>
       </c>
       <c r="AC7" s="1" t="n">
-        <v>46204.37858796296</v>
+        <v>46205.00364583333</v>
       </c>
       <c r="AD7" s="1" t="n">
-        <v>46204.56600694444</v>
+        <v>46205.06435185186</v>
       </c>
       <c r="AE7" t="n">
-        <v>16197</v>
-      </c>
-      <c r="AF7" t="inlineStr"/>
+        <v>5251</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>[2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1392,7 +1384,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8D6AA44A-CE22-48B1-8CED-5CBB40FBEE16</t>
+          <t>55CDBADD-FB23-4E6F-808F-30520080D01B</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1422,7 +1414,7 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
@@ -1454,12 +1446,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-6997-16-1</t>
+          <t>Honeywell7810PC-6997-4-1</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGNETICO PUERTA PASILLO CUARTO TECNICO CAJERO </t>
+          <t>INFRARROJO CUARTO AREA COMUN CAJERO</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -1492,7 +1484,7 @@
       </c>
       <c r="Y8" t="inlineStr"/>
       <c r="Z8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -1500,20 +1492,20 @@
         </is>
       </c>
       <c r="AB8" s="1" t="n">
-        <v>46205.00329861111</v>
+        <v>46205.00358796296</v>
       </c>
       <c r="AC8" s="1" t="n">
-        <v>46205.00336805556</v>
+        <v>46205.00364583333</v>
       </c>
       <c r="AD8" s="1" t="n">
         <v>46205.06435185186</v>
       </c>
       <c r="AE8" t="n">
-        <v>5275</v>
+        <v>5250</v>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>[2026-07-02 00:07:16] JUAN RODOLFO VASQUEZ ALZATE: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 00:07:24] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
+          <t>[2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1517,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0825C3AE-74CB-4CC0-867C-0E7C79C7FDE0</t>
+          <t>395B23B6-AD7D-4565-A9CE-5AFB32AF8C73</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1587,12 +1579,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-6997-2-1</t>
+          <t>Honeywell7810PC-6997-9-1</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>INFRARROJO ENTRADA HALL CAJERO</t>
+          <t xml:space="preserve">MAGNETICO PUERTA SALIDA EMERGENCIA 1 CAJERO </t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1633,20 +1625,20 @@
         </is>
       </c>
       <c r="AB9" s="1" t="n">
-        <v>46205.00351851852</v>
+        <v>46205.00359953703</v>
       </c>
       <c r="AC9" s="1" t="n">
-        <v>46205.00357638889</v>
+        <v>46205.0036574074</v>
       </c>
       <c r="AD9" s="1" t="n">
         <v>46205.06435185186</v>
       </c>
       <c r="AE9" t="n">
-        <v>5256</v>
+        <v>5249</v>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>[2026-07-02 00:05:34] JUAN RODOLFO VASQUEZ ALZATE: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 00:05:38] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVAN FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
+          <t>[2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1650,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9215F0DF-62AC-435C-8599-4FC8964BC185</t>
+          <t>C778A9A5-5563-4BD4-A8D6-9841322F6AA3</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1720,12 +1712,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-6997-12-1</t>
+          <t>Honeywell7810PC-6997-6-1</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>INFRARROJO PASILLO ATRAS CAJERO</t>
+          <t>INFRARROJO PASILLO SALIDA DE EMERGECIA 1 CAJERO</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1758,7 +1750,7 @@
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1766,16 +1758,16 @@
         </is>
       </c>
       <c r="AB10" s="1" t="n">
-        <v>46205.00357638889</v>
+        <v>46205.0037037037</v>
       </c>
       <c r="AC10" s="1" t="n">
-        <v>46205.00364583333</v>
+        <v>46205.00378472222</v>
       </c>
       <c r="AD10" s="1" t="n">
         <v>46205.06435185186</v>
       </c>
       <c r="AE10" t="n">
-        <v>5251</v>
+        <v>5240</v>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
@@ -1786,19 +1778,19 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0CF7D86D-118E-4E73-813B-DA90EB515E49</t>
+          <t>47CB88CB-13C7-4ADC-A6B5-C6AA3ADBA1D4</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>55CDBADD-FB23-4E6F-808F-30520080D01B</t>
+          <t>9D9CFC5D-06C5-476E-AC1D-BFC570DFF73B</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6997</v>
+        <v>8240</v>
       </c>
       <c r="D11" t="n">
-        <v>8726</v>
+        <v>4316</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1807,21 +1799,21 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SUR</t>
+          <t>BOG Y SABANA</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>CUNDINAMARCA</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CALI</t>
+          <t>BOGOTÁ, D.C.</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -1848,22 +1840,22 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>8726 8727 8728 8729 C MF HALL CALI PRINCIPAL - 6997 - AdminSUC - DIEBOLD</t>
+          <t>4316 C LA GRAN FERIA CAMPESINA - 8240 - TBS - DIEBOLD</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-6997-4-1</t>
+          <t>SGIII-8240-4-2</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>INFRARROJO CUARTO AREA COMUN CAJERO</t>
+          <t>MICROSUICHE FASCIA SUPERIOR CAJERO</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>SGIII</t>
         </is>
       </c>
       <c r="S11" t="n">
@@ -1871,27 +1863,23 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>JUAN RODOLFO VASQUEZ ALZATE</t>
+          <t>Jhon Fredy Ocampo Yepez</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>Falso positivo</t>
+          <t>Falso Positivo</t>
         </is>
       </c>
       <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>FUNCIONARIOS</t>
-        </is>
-      </c>
+      <c r="W11" t="inlineStr"/>
       <c r="X11">
         <f>EXACT(TRIM(UPPER(V11)), TRIM(UPPER(W11)))</f>
         <v/>
       </c>
       <c r="Y11" t="inlineStr"/>
       <c r="Z11" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1899,39 +1887,39 @@
         </is>
       </c>
       <c r="AB11" s="1" t="n">
-        <v>46205.00358796296</v>
+        <v>46205.48380787037</v>
       </c>
       <c r="AC11" s="1" t="n">
-        <v>46205.00364583333</v>
+        <v>46205.48390046296</v>
       </c>
       <c r="AD11" s="1" t="n">
-        <v>46205.06435185186</v>
+        <v>46205.55003472222</v>
       </c>
       <c r="AE11" t="n">
-        <v>5250</v>
+        <v>5722</v>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>[2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
+          <t>[2026-07-02 11:36:57] Jhon Fredy Ocampo Yepez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 13:11:01] Jhon Fredy Ocampo Yepez: Se verifica por video COMMAND , Todas las cámaras en tiempo real, se observa el SITIO en aparente normalidad y sin afectación alguna Se observa personal TECNICO DE DIEBOLD en el sitio || [2026-07-02 13:11:12] Jhon Fredy Ocampo Yepez: Mal manejo por desarme inoportuno</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0CF7D86D-118E-4E73-813B-DA90EB515E49</t>
+          <t>A8EC36AD-F179-46AC-8B2F-25BC1679025B</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>395B23B6-AD7D-4565-A9CE-5AFB32AF8C73</t>
+          <t>6B863118-F72D-4C86-A2D9-B5FA147CFC28</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>6997</v>
+        <v>9018</v>
       </c>
       <c r="D12" t="n">
-        <v>8726</v>
+        <v>2144</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1945,16 +1933,16 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>NARIÑO</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CALI</t>
+          <t>PASTO</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -1981,22 +1969,22 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>8726 8727 8728 8729 C MF HALL CALI PRINCIPAL - 6997 - AdminSUC - DIEBOLD</t>
+          <t>2144 4878 6895 C AVENIDA LOS ESTUDIANTES - 9018 - BK - DIEBOLD - NCR</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-6997-9-1</t>
+          <t>SGIII-9018-15-3</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGNETICO PUERTA SALIDA EMERGENCIA 1 CAJERO </t>
+          <t>MICROSUICH TAPA TECLADO CAJERO</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>SGIII</t>
         </is>
       </c>
       <c r="S12" t="n">
@@ -2004,18 +1992,18 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>JUAN RODOLFO VASQUEZ ALZATE</t>
+          <t>Laura Valentina Restrepo Jaramillo</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>Falso positivo</t>
+          <t>Falso Positivo</t>
         </is>
       </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr">
         <is>
-          <t>FUNCIONARIOS</t>
+          <t>BRINKS</t>
         </is>
       </c>
       <c r="X12">
@@ -2024,7 +2012,7 @@
       </c>
       <c r="Y12" t="inlineStr"/>
       <c r="Z12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -2032,39 +2020,39 @@
         </is>
       </c>
       <c r="AB12" s="1" t="n">
-        <v>46205.00359953703</v>
+        <v>46205.58280092593</v>
       </c>
       <c r="AC12" s="1" t="n">
-        <v>46205.0036574074</v>
+        <v>46205.58287037037</v>
       </c>
       <c r="AD12" s="1" t="n">
-        <v>46205.06435185186</v>
+        <v>46205.73596064815</v>
       </c>
       <c r="AE12" t="n">
-        <v>5249</v>
+        <v>13233</v>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
-          <t>[2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
+          <t>[2026-07-02 13:59:26] Laura Valentina Restrepo Jaramillo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 13:59:37] Laura Valentina Restrepo Jaramillo: ¡Enviando reacción correspondiente!  GAM -POLICIA  No carga video || [2026-07-02 14:19:51] Laura Valentina Restrepo Jaramillo: Se verifica por video cámara relacionada en tiempo real, TDV en el punto en aparente normalidad vatco || [2026-07-02 14:19:56] Laura Valentina Restrepo Jaramillo: Activación generada por desarme inoportuno</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0CF7D86D-118E-4E73-813B-DA90EB515E49</t>
+          <t>9DD6EA01-B5FD-494A-A04F-9A477C0544A0</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>C778A9A5-5563-4BD4-A8D6-9841322F6AA3</t>
+          <t>48D3E849-B16A-4966-A04F-8DDD7A2FF193</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>6997</v>
+        <v>8921</v>
       </c>
       <c r="D13" t="n">
-        <v>8726</v>
+        <v>7469</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2073,21 +2061,21 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SUR</t>
+          <t>CENTRO</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>META</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CALI</t>
+          <t>VILLAVICENCIO</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -2099,37 +2087,37 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
+          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>activación perimetral</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>activación perimetral atm</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>8726 8727 8728 8729 C MF HALL CALI PRINCIPAL - 6997 - AdminSUC - DIEBOLD</t>
+          <t>7469 4806 4807 C TOCORAGUA - 8921 - TBS - NCR</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Honeywell7810PC-6997-6-1</t>
+          <t>SGIII-8921-8-1</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>INFRARROJO PASILLO SALIDA DE EMERGECIA 1 CAJERO</t>
+          <t xml:space="preserve">TAMPER CENTRAL ALARMA CAJERO </t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Honeywell</t>
+          <t>SGIII</t>
         </is>
       </c>
       <c r="S13" t="n">
@@ -2137,18 +2125,18 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>JUAN RODOLFO VASQUEZ ALZATE</t>
+          <t>Neidy Martínez</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>Falso positivo</t>
+          <t>Falso Positivo</t>
         </is>
       </c>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr">
         <is>
-          <t>FUNCIONARIOS</t>
+          <t>TRANSBANK</t>
         </is>
       </c>
       <c r="X13">
@@ -2157,7 +2145,7 @@
       </c>
       <c r="Y13" t="inlineStr"/>
       <c r="Z13" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -2165,39 +2153,39 @@
         </is>
       </c>
       <c r="AB13" s="1" t="n">
-        <v>46205.0037037037</v>
+        <v>46205.598125</v>
       </c>
       <c r="AC13" s="1" t="n">
-        <v>46205.00378472222</v>
+        <v>46205.59818287037</v>
       </c>
       <c r="AD13" s="1" t="n">
-        <v>46205.06435185186</v>
+        <v>46205.77240740741</v>
       </c>
       <c r="AE13" t="n">
-        <v>5240</v>
+        <v>15058</v>
       </c>
       <c r="AF13" t="inlineStr">
         <is>
-          <t>[2026-07-02 00:06:57] JUAN RODOLFO VASQUEZ ALZATE: FUNCIONARIOS DE OBRAS EN EL SITIO || [2026-07-02 01:32:29] JUAN RODOLFO VASQUEZ ALZATE: SE VALIDA POR VIDEO COMMAND SE OBSERVA TDV TRANSBANK EN EL SITIO    SE GENERAN MALOS MANEJOS POR NO DESARME DE PARTICION</t>
+          <t>[2026-07-02 14:21:30] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 14:22:37] Neidy Martínez: Se valida por video command se observa USUARIO realizando transacción en el momento de la activación || [2026-07-02 14:23:05] Neidy Martínez: desarme de técnicos DIEBOLD en el sitio   Mal manejo, personal no realizan bypass de la zona de forma oportuna</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>47CB88CB-13C7-4ADC-A6B5-C6AA3ADBA1D4</t>
+          <t>66A1721F-9685-4A67-A14C-83CC3713A7D9</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>9D9CFC5D-06C5-476E-AC1D-BFC570DFF73B</t>
+          <t>D6D8DED2-9361-4132-B641-690F14368B77</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8240</v>
+        <v>8921</v>
       </c>
       <c r="D14" t="n">
-        <v>4316</v>
+        <v>7469</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2206,17 +2194,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>BOG Y SABANA</t>
+          <t>CENTRO</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>CUNDINAMARCA</t>
+          <t>META</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>BOGOTÁ, D.C.</t>
+          <t>VILLAVICENCIO</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -2247,17 +2235,17 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>4316 C LA GRAN FERIA CAMPESINA - 8240 - TBS - DIEBOLD</t>
+          <t>7469 4806 4807 C TOCORAGUA - 8921 - TBS - NCR</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>SGIII-8240-4-2</t>
+          <t>SGIII-8921-2-1</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>MICROSUICHE FASCIA SUPERIOR CAJERO</t>
+          <t xml:space="preserve">MAGNETICO CUARTO CAJEROS </t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -2270,7 +2258,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>Jhon Fredy Ocampo Yepez</t>
+          <t>Adier Cuitiva Mayo</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -2279,14 +2267,18 @@
         </is>
       </c>
       <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>TRANSBANK</t>
+        </is>
+      </c>
       <c r="X14">
         <f>EXACT(TRIM(UPPER(V14)), TRIM(UPPER(W14)))</f>
         <v/>
       </c>
       <c r="Y14" t="inlineStr"/>
       <c r="Z14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -2294,39 +2286,39 @@
         </is>
       </c>
       <c r="AB14" s="1" t="n">
-        <v>46205.48380787037</v>
+        <v>46205.60173611111</v>
       </c>
       <c r="AC14" s="1" t="n">
-        <v>46205.48390046296</v>
+        <v>46205.60180555555</v>
       </c>
       <c r="AD14" s="1" t="n">
-        <v>46205.55003472222</v>
+        <v>46205.62008101852</v>
       </c>
       <c r="AE14" t="n">
-        <v>5722</v>
+        <v>1585</v>
       </c>
       <c r="AF14" t="inlineStr">
         <is>
-          <t>[2026-07-02 11:36:57] Jhon Fredy Ocampo Yepez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 13:11:01] Jhon Fredy Ocampo Yepez: Se verifica por video COMMAND , Todas las cámaras en tiempo real, se observa el SITIO en aparente normalidad y sin afectación alguna Se observa personal TECNICO DE DIEBOLD en el sitio || [2026-07-02 13:11:12] Jhon Fredy Ocampo Yepez: Mal manejo por desarme inoportuno</t>
+          <t>[2026-07-02 14:26:40] Adier Cuitiva Mayo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 14:36:04] Adier Cuitiva Mayo: Se verifica por video cámara relacionada en tiempo real, TECNICO en aparente normalidad</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>A8EC36AD-F179-46AC-8B2F-25BC1679025B</t>
+          <t>66A1721F-9685-4A67-A14C-83CC3713A7D9</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6B863118-F72D-4C86-A2D9-B5FA147CFC28</t>
+          <t>DF3BDEFB-CDE3-492F-B007-6FCDFABE1CFB</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>9018</v>
+        <v>8921</v>
       </c>
       <c r="D15" t="n">
-        <v>2144</v>
+        <v>7469</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2335,21 +2327,21 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SUR</t>
+          <t>CENTRO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NARIÑO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>PASTO</t>
+          <t>VILLAVICENCIO</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
@@ -2361,32 +2353,32 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
+          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>activación perimetral</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>activación perimetral atm</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2144 4878 6895 C AVENIDA LOS ESTUDIANTES - 9018 - BK - DIEBOLD - NCR</t>
+          <t>7469 4806 4807 C TOCORAGUA - 8921 - TBS - NCR</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>SGIII-9018-15-3</t>
+          <t>SGIII-8921-6-1</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>MICROSUICH TAPA TECLADO CAJERO</t>
+          <t xml:space="preserve">TAMPER SISMICO CUARTO CAJEROS </t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -2399,7 +2391,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>Laura Valentina Restrepo Jaramillo</t>
+          <t>Adier Cuitiva Mayo</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2410,7 +2402,7 @@
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr">
         <is>
-          <t>BRINKS</t>
+          <t>TRANSBANK</t>
         </is>
       </c>
       <c r="X15">
@@ -2419,7 +2411,7 @@
       </c>
       <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -2427,32 +2419,28 @@
         </is>
       </c>
       <c r="AB15" s="1" t="n">
-        <v>46205.58280092593</v>
+        <v>46205.60268518519</v>
       </c>
       <c r="AC15" s="1" t="n">
-        <v>46205.58287037037</v>
+        <v>46205.60271990741</v>
       </c>
       <c r="AD15" s="1" t="n">
-        <v>46205.73596064815</v>
+        <v>46205.62008101852</v>
       </c>
       <c r="AE15" t="n">
-        <v>13233</v>
-      </c>
-      <c r="AF15" t="inlineStr">
-        <is>
-          <t>[2026-07-02 13:59:26] Laura Valentina Restrepo Jaramillo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 13:59:37] Laura Valentina Restrepo Jaramillo: ¡Enviando reacción correspondiente!  GAM -POLICIA  No carga video || [2026-07-02 14:19:51] Laura Valentina Restrepo Jaramillo: Se verifica por video cámara relacionada en tiempo real, TDV en el punto en aparente normalidad vatco || [2026-07-02 14:19:56] Laura Valentina Restrepo Jaramillo: Activación generada por desarme inoportuno</t>
-        </is>
-      </c>
+        <v>1503</v>
+      </c>
+      <c r="AF15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>9DD6EA01-B5FD-494A-A04F-9A477C0544A0</t>
+          <t>66A1721F-9685-4A67-A14C-83CC3713A7D9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>48D3E849-B16A-4966-A04F-8DDD7A2FF193</t>
+          <t>E89171C5-A464-4CE6-A483-0B947C6A1147</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -2482,7 +2470,7 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
         <v>1</v>
@@ -2494,17 +2482,17 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
+          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral atm</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2514,12 +2502,12 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>SGIII-8921-8-1</t>
+          <t>SGIII-8921-3-1</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMPER CENTRAL ALARMA CAJERO </t>
+          <t>INFRARROJO CUARTO CAJERO</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -2532,7 +2520,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>Neidy Martínez</t>
+          <t>Adier Cuitiva Mayo</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2552,7 +2540,7 @@
       </c>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -2560,22 +2548,18 @@
         </is>
       </c>
       <c r="AB16" s="1" t="n">
-        <v>46205.598125</v>
+        <v>46205.60274305556</v>
       </c>
       <c r="AC16" s="1" t="n">
-        <v>46205.59818287037</v>
+        <v>46205.6027662037</v>
       </c>
       <c r="AD16" s="1" t="n">
-        <v>46205.77240740741</v>
+        <v>46205.62008101852</v>
       </c>
       <c r="AE16" t="n">
-        <v>15058</v>
-      </c>
-      <c r="AF16" t="inlineStr">
-        <is>
-          <t>[2026-07-02 14:21:30] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 14:22:37] Neidy Martínez: Se valida por video command se observa USUARIO realizando transacción en el momento de la activación || [2026-07-02 14:23:05] Neidy Martínez: desarme de técnicos DIEBOLD en el sitio   Mal manejo, personal no realizan bypass de la zona de forma oportuna</t>
-        </is>
-      </c>
+        <v>1498</v>
+      </c>
+      <c r="AF16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2585,7 +2569,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>D6D8DED2-9361-4132-B641-690F14368B77</t>
+          <t>24E80F05-553C-491E-86E1-8F64E88DCA0E</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2615,7 +2599,7 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>1</v>
@@ -2627,17 +2611,17 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
+          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>activación perimetral</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>activación perimetral atm</t>
+          <t>activación tamper y antimascara</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2647,12 +2631,12 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>SGIII-8921-2-1</t>
+          <t>SGIII-8921-4-1</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGNETICO CUARTO CAJEROS </t>
+          <t xml:space="preserve">TAMPER Y ANTIMASCARA CUARTO CAJEROS </t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -2685,7 +2669,7 @@
       </c>
       <c r="Y17" t="inlineStr"/>
       <c r="Z17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -2693,32 +2677,28 @@
         </is>
       </c>
       <c r="AB17" s="1" t="n">
-        <v>46205.60173611111</v>
+        <v>46205.60290509259</v>
       </c>
       <c r="AC17" s="1" t="n">
-        <v>46205.60180555555</v>
+        <v>46205.60295138889</v>
       </c>
       <c r="AD17" s="1" t="n">
         <v>46205.62008101852</v>
       </c>
       <c r="AE17" t="n">
-        <v>1585</v>
-      </c>
-      <c r="AF17" t="inlineStr">
-        <is>
-          <t>[2026-07-02 14:26:40] Adier Cuitiva Mayo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 14:36:04] Adier Cuitiva Mayo: Se verifica por video cámara relacionada en tiempo real, TECNICO en aparente normalidad</t>
-        </is>
-      </c>
+        <v>1484</v>
+      </c>
+      <c r="AF17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>66A1721F-9685-4A67-A14C-83CC3713A7D9</t>
+          <t>1A312E74-19F2-4F11-86E2-6BDE2083FC21</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DF3BDEFB-CDE3-492F-B007-6FCDFABE1CFB</t>
+          <t>2E9367C4-B5FD-4341-A3B0-8F31B5F96452</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -2748,7 +2728,7 @@
         </is>
       </c>
       <c r="I18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
@@ -2760,17 +2740,17 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
+          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral atm</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2780,12 +2760,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>SGIII-8921-6-1</t>
+          <t>SGIII-8921-2-1</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMPER SISMICO CUARTO CAJEROS </t>
+          <t xml:space="preserve">MAGNETICO CUARTO CAJEROS </t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -2798,7 +2778,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>Adier Cuitiva Mayo</t>
+          <t>Laura Valentina Restrepo Jaramillo</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2818,7 +2798,7 @@
       </c>
       <c r="Y18" t="inlineStr"/>
       <c r="Z18" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -2826,35 +2806,39 @@
         </is>
       </c>
       <c r="AB18" s="1" t="n">
-        <v>46205.60268518519</v>
+        <v>46205.65268518519</v>
       </c>
       <c r="AC18" s="1" t="n">
-        <v>46205.60271990741</v>
+        <v>46205.65277777778</v>
       </c>
       <c r="AD18" s="1" t="n">
-        <v>46205.62008101852</v>
+        <v>46205.75859953704</v>
       </c>
       <c r="AE18" t="n">
-        <v>1503</v>
-      </c>
-      <c r="AF18" t="inlineStr"/>
+        <v>9151</v>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>[2026-07-02 15:40:40] Laura Valentina Restrepo Jaramillo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 15:40:49] Laura Valentina Restrepo Jaramillo: Se verifica por video cámara relacionada en tiempo real, TECNICO en aparente normalidad diebold</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>66A1721F-9685-4A67-A14C-83CC3713A7D9</t>
+          <t>E44254EE-15CD-41C9-9DB3-E9340C29C9ED</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>E89171C5-A464-4CE6-A483-0B947C6A1147</t>
+          <t>A4E4DB68-41FC-4BB1-B722-411E9874FB6E</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>8921</v>
+        <v>9060</v>
       </c>
       <c r="D19" t="n">
-        <v>7469</v>
+        <v>2988</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2863,21 +2847,21 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>SUR</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>VILLAVICENCIO</t>
+          <t>CALI</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -2904,17 +2888,17 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>7469 4806 4807 C TOCORAGUA - 8921 - TBS - NCR</t>
+          <t>2988 C PARQUE DE LA CAÑA S - 9060 - TBS - NCR</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>SGIII-8921-3-1</t>
+          <t>SGIII-9060-7-2</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>INFRARROJO CUARTO CAJERO</t>
+          <t>MICROSUICHE DIAL COFRE CAJERO</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2927,18 +2911,18 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>Adier Cuitiva Mayo</t>
+          <t>ARELY TORRES</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Falso Positivo</t>
+          <t>Falso positivo</t>
         </is>
       </c>
       <c r="V19" t="inlineStr"/>
       <c r="W19" t="inlineStr">
         <is>
-          <t>TRANSBANK</t>
+          <t>BRINKS</t>
         </is>
       </c>
       <c r="X19">
@@ -2947,7 +2931,7 @@
       </c>
       <c r="Y19" t="inlineStr"/>
       <c r="Z19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -2955,35 +2939,39 @@
         </is>
       </c>
       <c r="AB19" s="1" t="n">
-        <v>46205.60274305556</v>
+        <v>46206.29728009259</v>
       </c>
       <c r="AC19" s="1" t="n">
-        <v>46205.6027662037</v>
+        <v>46206.29736111111</v>
       </c>
       <c r="AD19" s="1" t="n">
-        <v>46205.62008101852</v>
+        <v>46206.39796296296</v>
       </c>
       <c r="AE19" t="n">
-        <v>1498</v>
-      </c>
-      <c r="AF19" t="inlineStr"/>
+        <v>8699</v>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>[2026-07-03 07:08:21] ARELY TORRES: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ || [2026-07-03 07:08:21] ARELY TORRES: [SOP:3] Documentando ✅ || [2026-07-03 07:09:00] ARELY TORRES: SE GENERA COBRO DE MALOS, ZONA SIN BYPASEAR A TIEMPO Se valida video por Command y no se evidencia novedad. TDV EN SITIO || [2026-07-03 07:09:01] ARELY TORRES: BK</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>66A1721F-9685-4A67-A14C-83CC3713A7D9</t>
+          <t>E44254EE-15CD-41C9-9DB3-E9340C29C9ED</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>24E80F05-553C-491E-86E1-8F64E88DCA0E</t>
+          <t>FF7E0E5D-E05E-41EF-85BD-43BB04DE8CC1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>8921</v>
+        <v>9060</v>
       </c>
       <c r="D20" t="n">
-        <v>7469</v>
+        <v>2988</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2992,17 +2980,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>SUR</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>VALLE DEL CAUCA</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>VILLAVICENCIO</t>
+          <t>CALI</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -3018,32 +3006,32 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
+          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>activación tamper y antimascara</t>
+          <t>activación perimetral atm</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>7469 4806 4807 C TOCORAGUA - 8921 - TBS - NCR</t>
+          <t>2988 C PARQUE DE LA CAÑA S - 9060 - TBS - NCR</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>SGIII-8921-4-1</t>
+          <t>SGIII-9060-9-2</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAMPER Y ANTIMASCARA CUARTO CAJEROS </t>
+          <t>MAGNETICO COFRE CAJERO</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -3056,18 +3044,18 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>Adier Cuitiva Mayo</t>
+          <t>ARELY TORRES</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Falso Positivo</t>
+          <t>Falso positivo</t>
         </is>
       </c>
       <c r="V20" t="inlineStr"/>
       <c r="W20" t="inlineStr">
         <is>
-          <t>TRANSBANK</t>
+          <t>BRINKS</t>
         </is>
       </c>
       <c r="X20">
@@ -3076,7 +3064,7 @@
       </c>
       <c r="Y20" t="inlineStr"/>
       <c r="Z20" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -3084,35 +3072,35 @@
         </is>
       </c>
       <c r="AB20" s="1" t="n">
-        <v>46205.60290509259</v>
+        <v>46206.29730324074</v>
       </c>
       <c r="AC20" s="1" t="n">
-        <v>46205.60295138889</v>
+        <v>46206.29738425926</v>
       </c>
       <c r="AD20" s="1" t="n">
-        <v>46205.62008101852</v>
+        <v>46206.39796296296</v>
       </c>
       <c r="AE20" t="n">
-        <v>1484</v>
+        <v>8697</v>
       </c>
       <c r="AF20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>1A312E74-19F2-4F11-86E2-6BDE2083FC21</t>
+          <t>7059BA0F-9CDF-47B9-91E3-79EA472C375C</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2E9367C4-B5FD-4341-A3B0-8F31B5F96452</t>
+          <t>9E33C3F6-7EB1-45A5-8215-A8BC637490A5</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>8921</v>
+        <v>6023</v>
       </c>
       <c r="D21" t="n">
-        <v>7469</v>
+        <v>1055</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3121,21 +3109,21 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>CENTRO</t>
+          <t>ANTIOQUIA</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>ANTIOQUIA</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>VILLAVICENCIO</t>
+          <t>MEDELLÍN</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
@@ -3162,17 +3150,17 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>7469 4806 4807 C TOCORAGUA - 8921 - TBS - NCR</t>
+          <t>1055 1056 1057 C HALL FLORIDA PARQUE - 6023</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>SGIII-8921-2-1</t>
+          <t>SGIII-6023-14-2</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAGNETICO CUARTO CAJEROS </t>
+          <t>MICROSUICHE FASCIA INFERIOR KIOSCO</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -3185,18 +3173,18 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>Laura Valentina Restrepo Jaramillo</t>
+          <t>kelly aguirre</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Falso Positivo</t>
+          <t xml:space="preserve">Falso positivo </t>
         </is>
       </c>
       <c r="V21" t="inlineStr"/>
       <c r="W21" t="inlineStr">
         <is>
-          <t>TRANSBANK</t>
+          <t>FUNCIONARIOS</t>
         </is>
       </c>
       <c r="X21">
@@ -3205,7 +3193,7 @@
       </c>
       <c r="Y21" t="inlineStr"/>
       <c r="Z21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -3213,39 +3201,35 @@
         </is>
       </c>
       <c r="AB21" s="1" t="n">
-        <v>46205.65268518519</v>
+        <v>46207.68248842593</v>
       </c>
       <c r="AC21" s="1" t="n">
-        <v>46205.65277777778</v>
+        <v>46207.68256944444</v>
       </c>
       <c r="AD21" s="1" t="n">
-        <v>46205.75859953704</v>
+        <v>46207.69075231482</v>
       </c>
       <c r="AE21" t="n">
-        <v>9151</v>
-      </c>
-      <c r="AF21" t="inlineStr">
-        <is>
-          <t>[2026-07-02 15:40:40] Laura Valentina Restrepo Jaramillo: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-02 15:40:49] Laura Valentina Restrepo Jaramillo: Se verifica por video cámara relacionada en tiempo real, TECNICO en aparente normalidad diebold</t>
-        </is>
-      </c>
+        <v>714</v>
+      </c>
+      <c r="AF21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E44254EE-15CD-41C9-9DB3-E9340C29C9ED</t>
+          <t>D44BDE4D-3C6E-462C-A838-D9BDF2DB8EF1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>A4E4DB68-41FC-4BB1-B722-411E9874FB6E</t>
+          <t>4287379F-8B0B-47AF-9246-9F878359E816</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>9060</v>
+        <v>7653</v>
       </c>
       <c r="D22" t="n">
-        <v>2988</v>
+        <v>6628</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3254,17 +3238,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SUR</t>
+          <t>BOG Y SABANA</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>CUNDINAMARCA</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CALI</t>
+          <t>MOSQUERA</t>
         </is>
       </c>
       <c r="I22" t="n">
@@ -3295,17 +3279,17 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2988 C PARQUE DE LA CAÑA S - 9060 - TBS - NCR</t>
+          <t>6628 C MULTIFUNCIONAL MOSQUERA - 7653 - AdminSUC</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>SGIII-9060-7-2</t>
+          <t>SGIII-7653-11-2</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>MICROSUICHE DIAL COFRE CAJERO</t>
+          <t xml:space="preserve">MAGNETICO COFRE CJAERO </t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -3318,7 +3302,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>ARELY TORRES</t>
+          <t>Neidy Martínez</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -3329,7 +3313,7 @@
       <c r="V22" t="inlineStr"/>
       <c r="W22" t="inlineStr">
         <is>
-          <t>BRINKS</t>
+          <t>FUNCIONARIOS</t>
         </is>
       </c>
       <c r="X22">
@@ -3338,7 +3322,7 @@
       </c>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -3346,39 +3330,39 @@
         </is>
       </c>
       <c r="AB22" s="1" t="n">
-        <v>46206.29728009259</v>
+        <v>46213.26283564815</v>
       </c>
       <c r="AC22" s="1" t="n">
-        <v>46206.29736111111</v>
+        <v>46213.26297453704</v>
       </c>
       <c r="AD22" s="1" t="n">
-        <v>46206.39796296296</v>
+        <v>46213.44462962963</v>
       </c>
       <c r="AE22" t="n">
-        <v>8699</v>
+        <v>15707</v>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
-          <t>[2026-07-03 07:08:21] ARELY TORRES: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ || [2026-07-03 07:08:21] ARELY TORRES: [SOP:3] Documentando ✅ || [2026-07-03 07:09:00] ARELY TORRES: SE GENERA COBRO DE MALOS, ZONA SIN BYPASEAR A TIEMPO Se valida video por Command y no se evidencia novedad. TDV EN SITIO || [2026-07-03 07:09:01] ARELY TORRES: BK</t>
+          <t>[2026-07-10 06:19:27] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-10 06:20:09] Neidy Martínez: sin video || [2026-07-10 06:20:54] Neidy Martínez: 10/07/2026 06:20:00 S01011[#7653|Nri2/OP0022/OR0022]_x0014_ Partición Desarmada USUARIO  22 VATCO || [2026-07-10 06:21:07] Neidy Martínez: Mal manejo, personal en sitio no realiza desarme de la partición de forma oportuna</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E44254EE-15CD-41C9-9DB3-E9340C29C9ED</t>
+          <t>FAA6FA10-0FB6-47F7-8B2B-80AC373C2FA3</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>FF7E0E5D-E05E-41EF-85BD-43BB04DE8CC1</t>
+          <t>D0705EFA-4C24-4253-84E9-FE31929F07DB</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9060</v>
+        <v>7482</v>
       </c>
       <c r="D23" t="n">
-        <v>2988</v>
+        <v>7121</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3387,17 +3371,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SUR</t>
+          <t>BOG Y SABANA</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>VALLE DEL CAUCA</t>
+          <t>CUNDINAMARCA</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>CALI</t>
+          <t>BOGOTÁ, D.C.</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -3428,22 +3412,22 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2988 C PARQUE DE LA CAÑA S - 9060 - TBS - NCR</t>
+          <t>7121 C MULTIFUNCIONAL PLAZA CLARO - 7482 - ATL - DIEBOLD</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>SGIII-9060-9-2</t>
+          <t>Honeywell7810PC-7482-54-2</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>MAGNETICO COFRE CAJERO</t>
+          <t xml:space="preserve">MAGNETICO CONTRATAPA INFERIOR CAJERO </t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>SGIII</t>
+          <t>Honeywell</t>
         </is>
       </c>
       <c r="S23" t="n">
@@ -3451,7 +3435,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>ARELY TORRES</t>
+          <t>JHON DAIRO ESCOBAR GARCIA</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -3462,7 +3446,7 @@
       <c r="V23" t="inlineStr"/>
       <c r="W23" t="inlineStr">
         <is>
-          <t>BRINKS</t>
+          <t>ATLAS</t>
         </is>
       </c>
       <c r="X23">
@@ -3471,7 +3455,7 @@
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
@@ -3479,1622 +3463,18 @@
         </is>
       </c>
       <c r="AB23" s="1" t="n">
-        <v>46206.29730324074</v>
+        <v>46216.26837962963</v>
       </c>
       <c r="AC23" s="1" t="n">
-        <v>46206.29738425926</v>
+        <v>46216.26842592593</v>
       </c>
       <c r="AD23" s="1" t="n">
-        <v>46206.39796296296</v>
+        <v>46216.47231481481</v>
       </c>
       <c r="AE23" t="n">
-        <v>8697</v>
+        <v>17620</v>
       </c>
       <c r="AF23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>7059BA0F-9CDF-47B9-91E3-79EA472C375C</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>9E33C3F6-7EB1-45A5-8215-A8BC637490A5</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>6023</v>
-      </c>
-      <c r="D24" t="n">
-        <v>1055</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>ANTIOQUIA</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>ANTIOQUIA</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>MEDELLÍN</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="n">
-        <v>1</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>1055 1056 1057 C HALL FLORIDA PARQUE - 6023</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>SGIII-6023-14-2</t>
-        </is>
-      </c>
-      <c r="Q24" t="inlineStr">
-        <is>
-          <t>MICROSUICHE FASCIA INFERIOR KIOSCO</t>
-        </is>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S24" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>kelly aguirre</t>
-        </is>
-      </c>
-      <c r="U24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Falso positivo </t>
-        </is>
-      </c>
-      <c r="V24" t="inlineStr"/>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24">
-        <f>EXACT(TRIM(UPPER(V24)), TRIM(UPPER(W24)))</f>
-        <v/>
-      </c>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="n">
-        <v>7</v>
-      </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB24" s="1" t="n">
-        <v>46207.68248842593</v>
-      </c>
-      <c r="AC24" s="1" t="n">
-        <v>46207.68256944444</v>
-      </c>
-      <c r="AD24" s="1" t="n">
-        <v>46207.69075231482</v>
-      </c>
-      <c r="AE24" t="n">
-        <v>714</v>
-      </c>
-      <c r="AF24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>CA89E80A-B81C-4C07-A5A2-7D23EE987E16</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>D326EFA3-9528-458A-A0BD-38F0A8A05EEB</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>5494</v>
-      </c>
-      <c r="D25" t="n">
-        <v>1126</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>BOGOTÁ D.C.</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>1126 C HALL CC GRAN PLAZA BOSA - 5494</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>SGIII-5494-56-8</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>MAGNETICO FASCIA SUPERIOR CAJERO</t>
-        </is>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S25" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>JHON DAIRO ESCOBAR GARCIA</t>
-        </is>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>Mal manejo (Reacción)</t>
-        </is>
-      </c>
-      <c r="V25" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25">
-        <f>EXACT(TRIM(UPPER(V25)), TRIM(UPPER(W25)))</f>
-        <v/>
-      </c>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB25" s="1" t="n">
-        <v>46211.59497685185</v>
-      </c>
-      <c r="AC25" s="1" t="n">
-        <v>46211.59506944445</v>
-      </c>
-      <c r="AD25" s="1" t="n">
-        <v>46211.62721064815</v>
-      </c>
-      <c r="AE25" t="n">
-        <v>2785</v>
-      </c>
-      <c r="AF25" t="inlineStr">
-        <is>
-          <t>[2026-07-08 14:17:30] JHON DAIRO ESCOBAR GARCIA: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-08 14:18:01] JHON DAIRO ESCOBAR GARCIA: 8/7/2026, 2:16:43 p. m. SGIII-5494-8 CL Particion armada 61 Sin verificación de - Reporte de Cierre Normal - 61 ATLAS 1126 C HALL CC GRAN PLAZA BOSA - 5494 PARTICION 8 || [2026-07-08 14:23:56] JHON DAIRO ESCOBAR GARCIA: CRISTIAN DAVID PULIDO VANEGAS  GAM - 1.077.320.514 Disponible  3502477877 || [2026-07-08 14:24:28] JHON DAIRO ESCOBAR GARCIA: Enterado || [2026-07-08 15:02:49] JUAN RODOLFO VASQUEZ ALZATE: GAM JOHN HUERTAS  PASA REVISTA ENCUENTRA PERSONAL DE TDV ATLAS EN SERVICIO TECNICO TODO BIEN CERRADO Y AJUSTADO, OPERATIVO, ENERGIA ESTABLE, SIN SEÑALES DE VANDALISMO, SIN OLORES NI RUIDOS EXTRAÑOS, SIN OBRAS ALEDAÑAS, ALREDEDORES Y PERIMETRO SIN NOVEDAD, EL RESTO N2 A LA HORA</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>CA89E80A-B81C-4C07-A5A2-7D23EE987E16</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>9958268A-4787-434D-8421-DBCC5A407D01</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>5494</v>
-      </c>
-      <c r="D26" t="n">
-        <v>1126</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>BOGOTÁ D.C.</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="n">
-        <v>1</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>1126 C HALL CC GRAN PLAZA BOSA - 5494</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>SGIII-5494-55-8</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>MAGNETICO CONTRATAPA INFERIOR CAJERO</t>
-        </is>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S26" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>JHON DAIRO ESCOBAR GARCIA</t>
-        </is>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>Mal manejo (Reacción)</t>
-        </is>
-      </c>
-      <c r="V26" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26">
-        <f>EXACT(TRIM(UPPER(V26)), TRIM(UPPER(W26)))</f>
-        <v/>
-      </c>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="n">
-        <v>9</v>
-      </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB26" s="1" t="n">
-        <v>46211.59520833333</v>
-      </c>
-      <c r="AC26" s="1" t="n">
-        <v>46211.5953125</v>
-      </c>
-      <c r="AD26" s="1" t="n">
-        <v>46211.62637731482</v>
-      </c>
-      <c r="AE26" t="n">
-        <v>2693</v>
-      </c>
-      <c r="AF26" t="inlineStr">
-        <is>
-          <t>[2026-07-08 15:00:14] JUAN RODOLFO VASQUEZ ALZATE: GAM JOHN HUERTAS  PASA REVISTA ENCUENTRA PERSONAL DE TDV ATLAS EN SERVICIO TECNICO TODO BIEN CERRADO Y AJUSTADO, OPERATIVO, ENERGIA ESTABLE, SIN SEÑALES DE VANDALISMO, SIN OLORES NI RUIDOS EXTRAÑOS, SIN OBRAS ALEDAÑAS, ALREDEDORES Y PERIMETRO SIN NOVEDAD, EL RESTO N2 A LA HORA</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>CA89E80A-B81C-4C07-A5A2-7D23EE987E16</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>C9DB836E-56CB-4012-96E2-D4A44846539A</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>5494</v>
-      </c>
-      <c r="D27" t="n">
-        <v>1126</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>BOGOTÁ D.C.</t>
-        </is>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>1</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L27" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>1126 C HALL CC GRAN PLAZA BOSA - 5494</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>SGIII-5494-57-8</t>
-        </is>
-      </c>
-      <c r="Q27" t="inlineStr">
-        <is>
-          <t>MICROSUICHE DIAL COFRE CAJERO</t>
-        </is>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S27" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>JHON DAIRO ESCOBAR GARCIA</t>
-        </is>
-      </c>
-      <c r="U27" t="inlineStr">
-        <is>
-          <t>Mal manejo (Reacción)</t>
-        </is>
-      </c>
-      <c r="V27" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27">
-        <f>EXACT(TRIM(UPPER(V27)), TRIM(UPPER(W27)))</f>
-        <v/>
-      </c>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB27" s="1" t="n">
-        <v>46211.5978587963</v>
-      </c>
-      <c r="AC27" s="1" t="n">
-        <v>46211.5979050926</v>
-      </c>
-      <c r="AD27" s="1" t="n">
-        <v>46211.62666666666</v>
-      </c>
-      <c r="AE27" t="n">
-        <v>2489</v>
-      </c>
-      <c r="AF27" t="inlineStr">
-        <is>
-          <t>[2026-07-08 15:02:11] JUAN RODOLFO VASQUEZ ALZATE: GAM JOHN HUERTAS  PASA REVISTA ENCUENTRA PERSONAL DE TDV ATLAS EN SERVICIO TECNICO TODO BIEN CERRADO Y AJUSTADO, OPERATIVO, ENERGIA ESTABLE, SIN SEÑALES DE VANDALISMO, SIN OLORES NI RUIDOS EXTRAÑOS, SIN OBRAS ALEDAÑAS, ALREDEDORES Y PERIMETRO SIN NOVEDAD, EL RESTO N2 A LA HORA</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>CA89E80A-B81C-4C07-A5A2-7D23EE987E16</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>E7BF55E9-5EFB-4B67-9B87-FA5BCF9333BC</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>5494</v>
-      </c>
-      <c r="D28" t="n">
-        <v>1126</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>BOGOTÁ D.C.</t>
-        </is>
-      </c>
-      <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="n">
-        <v>1</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>1126 C HALL CC GRAN PLAZA BOSA - 5494</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>SGIII-5494-58-8</t>
-        </is>
-      </c>
-      <c r="Q28" t="inlineStr">
-        <is>
-          <t>MAGNETICO COFRE CAJERO</t>
-        </is>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S28" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>JHON DAIRO ESCOBAR GARCIA</t>
-        </is>
-      </c>
-      <c r="U28" t="inlineStr">
-        <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V28" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28">
-        <f>EXACT(TRIM(UPPER(V28)), TRIM(UPPER(W28)))</f>
-        <v/>
-      </c>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="n">
-        <v>8</v>
-      </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB28" s="1" t="n">
-        <v>46211.59789351852</v>
-      </c>
-      <c r="AC28" s="1" t="n">
-        <v>46211.59798611111</v>
-      </c>
-      <c r="AD28" s="1" t="n">
-        <v>46211.62690972222</v>
-      </c>
-      <c r="AE28" t="n">
-        <v>2507</v>
-      </c>
-      <c r="AF28" t="inlineStr">
-        <is>
-          <t>[2026-07-08 15:02:31] JUAN RODOLFO VASQUEZ ALZATE: GAM JOHN HUERTAS  PASA REVISTA ENCUENTRA PERSONAL DE TDV ATLAS EN SERVICIO TECNICO TODO BIEN CERRADO Y AJUSTADO, OPERATIVO, ENERGIA ESTABLE, SIN SEÑALES DE VANDALISMO, SIN OLORES NI RUIDOS EXTRAÑOS, SIN OBRAS ALEDAÑAS, ALREDEDORES Y PERIMETRO SIN NOVEDAD, EL RESTO N2 A LA HORA</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>D44BDE4D-3C6E-462C-A838-D9BDF2DB8EF1</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>4287379F-8B0B-47AF-9246-9F878359E816</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>7653</v>
-      </c>
-      <c r="D29" t="n">
-        <v>6628</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>MOSQUERA</t>
-        </is>
-      </c>
-      <c r="I29" t="n">
-        <v>1</v>
-      </c>
-      <c r="J29" t="n">
-        <v>1</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>6628 C MULTIFUNCIONAL MOSQUERA - 7653 - AdminSUC</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>SGIII-7653-11-2</t>
-        </is>
-      </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MAGNETICO COFRE CJAERO </t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S29" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>Neidy Martínez</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>Falso positivo</t>
-        </is>
-      </c>
-      <c r="V29" t="inlineStr"/>
-      <c r="W29" t="inlineStr">
-        <is>
-          <t>FUNCIONARIOS</t>
-        </is>
-      </c>
-      <c r="X29">
-        <f>EXACT(TRIM(UPPER(V29)), TRIM(UPPER(W29)))</f>
-        <v/>
-      </c>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="n">
-        <v>12</v>
-      </c>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB29" s="1" t="n">
-        <v>46213.26283564815</v>
-      </c>
-      <c r="AC29" s="1" t="n">
-        <v>46213.26297453704</v>
-      </c>
-      <c r="AD29" s="1" t="n">
-        <v>46213.44462962963</v>
-      </c>
-      <c r="AE29" t="n">
-        <v>15707</v>
-      </c>
-      <c r="AF29" t="inlineStr">
-        <is>
-          <t>[2026-07-10 06:19:27] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-10 06:20:09] Neidy Martínez: sin video || [2026-07-10 06:20:54] Neidy Martínez: 10/07/2026 06:20:00 S01011[#7653|Nri2/OP0022/OR0022]_x0014_ Partición Desarmada USUARIO  22 VATCO || [2026-07-10 06:21:07] Neidy Martínez: Mal manejo, personal en sitio no realiza desarme de la partición de forma oportuna</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>2C0EEBD4-6820-41B4-85BE-9AC2399B9127</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>71E4FC4F-EDDC-49E4-9D2C-0A2AE47C7903</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>7866</v>
-      </c>
-      <c r="D30" t="n">
-        <v>2054</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>SUR</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>RISARALDA</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>PEREIRA</t>
-        </is>
-      </c>
-      <c r="I30" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>8060 C EXITO PEREIRA CUARTO S - 7866 - TBS - DIEBOLD</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>SGIII-7866-2-1</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>MICROSUICHE TAPA TECLADO CUARTO TECNICO</t>
-        </is>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S30" t="n">
-        <v>0</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>Neidy Martínez</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V30" t="inlineStr">
-        <is>
-          <t>NCR</t>
-        </is>
-      </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>DIEBOLD</t>
-        </is>
-      </c>
-      <c r="X30">
-        <f>EXACT(TRIM(UPPER(V30)), TRIM(UPPER(W30)))</f>
-        <v/>
-      </c>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="n">
-        <v>7</v>
-      </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB30" s="1" t="n">
-        <v>46213.33342592593</v>
-      </c>
-      <c r="AC30" s="1" t="n">
-        <v>46213.33350694444</v>
-      </c>
-      <c r="AD30" s="1" t="n">
-        <v>46213.4652662037</v>
-      </c>
-      <c r="AE30" t="n">
-        <v>11391</v>
-      </c>
-      <c r="AF30" t="inlineStr">
-        <is>
-          <t>[2026-07-10 08:06:12] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-10 08:06:49] Neidy Martínez: Se valida por video command se observan TÉCNICOS NCR en el sitio   Mal manejo, personal no realizan bypass de la zona de forma oportuna</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>95E5AD83-983F-4872-BC44-8A2E3429E926</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>61F4ACA3-B50F-4C54-89A0-9A436CEF04E8</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>6904</v>
-      </c>
-      <c r="D31" t="n">
-        <v>4697</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>ANTIOQUIA</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>ANTIOQUIA</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>BELLO</t>
-        </is>
-      </c>
-      <c r="I31" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" t="n">
-        <v>1</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>WF 1055 - ZO09-Zonas 24H-Tamper y Antimascara AP:A</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>activación tamper y antimascara</t>
-        </is>
-      </c>
-      <c r="N31" t="inlineStr">
-        <is>
-          <t>activación tamper y antimascara</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>8507 8508 5022 6766 C CENTRO PAGOS BELLO - 6904 - TBS - DIEBOLD</t>
-        </is>
-      </c>
-      <c r="P31" t="inlineStr">
-        <is>
-          <t>Honeywell7810PC-6904-8-2</t>
-        </is>
-      </c>
-      <c r="Q31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAMPER CENTRAL ALARMA CAJERO </t>
-        </is>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Honeywell</t>
-        </is>
-      </c>
-      <c r="S31" t="n">
-        <v>1</v>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>Neidy Martínez</t>
-        </is>
-      </c>
-      <c r="U31" t="inlineStr">
-        <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V31" t="inlineStr">
-        <is>
-          <t>NCR</t>
-        </is>
-      </c>
-      <c r="W31" t="inlineStr">
-        <is>
-          <t>DIEBOLD</t>
-        </is>
-      </c>
-      <c r="X31">
-        <f>EXACT(TRIM(UPPER(V31)), TRIM(UPPER(W31)))</f>
-        <v/>
-      </c>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB31" s="1" t="n">
-        <v>46213.34752314815</v>
-      </c>
-      <c r="AC31" s="1" t="n">
-        <v>46213.34755787037</v>
-      </c>
-      <c r="AD31" s="1" t="n">
-        <v>46213.50226851852</v>
-      </c>
-      <c r="AE31" t="n">
-        <v>13370</v>
-      </c>
-      <c r="AF31" t="inlineStr">
-        <is>
-          <t>[2026-07-10 08:43:10] Neidy Martínez: [SOP:1] Validando Video ✅ [SOP:2] Enviando Reacción ✅ [SOP:3] Documentando ✅ || [2026-07-10 08:46:50] Neidy Martínez: Se valida por video command se observan TÉCNICOS NCR en el sitio   Mal manejo, personal no realizan bypass de la zona de forma oportuna</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>F52805E4-F45F-4D77-8EFE-7957327E7CEB</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>461A433F-2400-49BB-AA90-3F64CA9A4225</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>7946</v>
-      </c>
-      <c r="D32" t="n">
-        <v>5077</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>BOGOTÁ, D.C.</t>
-        </is>
-      </c>
-      <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="n">
-        <v>3</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>WF 1002 - AP03-Dia-No User In Data Base -  - UsuarioDesconocido</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>apertura por usuario desconocido</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>apertura por usuario desconocido (d)</t>
-        </is>
-      </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>5489 C CP UNICENTRO BOGOTA - 7946 - AdminSUC - BELLTECH -Mtto</t>
-        </is>
-      </c>
-      <c r="P32" t="inlineStr">
-        <is>
-          <t>SGIII-7946-2</t>
-        </is>
-      </c>
-      <c r="Q32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARTICION 2 </t>
-        </is>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S32" t="n">
-        <v>0</v>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>Jhon Fredy Ocampo Yepez</t>
-        </is>
-      </c>
-      <c r="U32" t="inlineStr">
-        <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V32" t="inlineStr">
-        <is>
-          <t>BRINKS</t>
-        </is>
-      </c>
-      <c r="W32" t="inlineStr">
-        <is>
-          <t>FUNCIONARIOS</t>
-        </is>
-      </c>
-      <c r="X32">
-        <f>EXACT(TRIM(UPPER(V32)), TRIM(UPPER(W32)))</f>
-        <v/>
-      </c>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB32" s="1" t="n">
-        <v>46214.46444444444</v>
-      </c>
-      <c r="AC32" s="1" t="n">
-        <v>46214.46445601852</v>
-      </c>
-      <c r="AD32" s="1" t="n">
-        <v>46214.47326388889</v>
-      </c>
-      <c r="AE32" t="n">
-        <v>762</v>
-      </c>
-      <c r="AF32" t="inlineStr">
-        <is>
-          <t>[2026-07-11 11:13:19] Jhon Fredy Ocampo Yepez: Mal manejo por no desarme de particion</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>F52805E4-F45F-4D77-8EFE-7957327E7CEB</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>37CEACE6-DCD5-49F8-B2AE-1169770F4179</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>7946</v>
-      </c>
-      <c r="D33" t="n">
-        <v>7980</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>BOGOTÁ, D.C.</t>
-        </is>
-      </c>
-      <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="n">
-        <v>3</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>WF 1002 - AP03-Dia-No User In Data Base -  - UsuarioDesconocido</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>apertura por usuario desconocido</t>
-        </is>
-      </c>
-      <c r="N33" t="inlineStr">
-        <is>
-          <t>apertura por usuario desconocido (d)</t>
-        </is>
-      </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>5489 C CP UNICENTRO BOGOTA - 7946 - AdminSUC - BELLTECH -Mtto</t>
-        </is>
-      </c>
-      <c r="P33" t="inlineStr">
-        <is>
-          <t>SGIII-7946-4</t>
-        </is>
-      </c>
-      <c r="Q33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARTICION 4 </t>
-        </is>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S33" t="n">
-        <v>1</v>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>Jhon Fredy Ocampo Yepez</t>
-        </is>
-      </c>
-      <c r="U33" t="inlineStr">
-        <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V33" t="inlineStr">
-        <is>
-          <t>BRINKS</t>
-        </is>
-      </c>
-      <c r="W33" t="inlineStr">
-        <is>
-          <t>FUNCIONARIOS</t>
-        </is>
-      </c>
-      <c r="X33">
-        <f>EXACT(TRIM(UPPER(V33)), TRIM(UPPER(W33)))</f>
-        <v/>
-      </c>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA33" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB33" s="1" t="n">
-        <v>46214.46508101852</v>
-      </c>
-      <c r="AC33" s="1" t="n">
-        <v>46214.4650925926</v>
-      </c>
-      <c r="AD33" s="1" t="n">
-        <v>46214.47326388889</v>
-      </c>
-      <c r="AE33" t="n">
-        <v>707</v>
-      </c>
-      <c r="AF33" t="inlineStr">
-        <is>
-          <t>[2026-07-11 11:13:19] Jhon Fredy Ocampo Yepez: Mal manejo por no desarme de particion</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>F52805E4-F45F-4D77-8EFE-7957327E7CEB</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>405E8895-3EC9-4A4E-AFB5-A0332577A1D5</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>7946</v>
-      </c>
-      <c r="D34" t="n">
-        <v>5077</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>BOGOTÁ, D.C.</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="n">
-        <v>3</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Baja</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>WF 1002 - AP03-Dia-No User In Data Base -  - UsuarioDesconocido</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>apertura por usuario desconocido</t>
-        </is>
-      </c>
-      <c r="N34" t="inlineStr">
-        <is>
-          <t>apertura por usuario desconocido (d)</t>
-        </is>
-      </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>5489 7980 C MULTIFUNCIONAL CP UNICENTRO BOGOTA SUC - 7946 - AdminSUC - BELLTECH -Mtto</t>
-        </is>
-      </c>
-      <c r="P34" t="inlineStr">
-        <is>
-          <t>SGIII-7946-1</t>
-        </is>
-      </c>
-      <c r="Q34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PARTICION 1 </t>
-        </is>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>SGIII</t>
-        </is>
-      </c>
-      <c r="S34" t="n">
-        <v>0</v>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>Jhon Fredy Ocampo Yepez</t>
-        </is>
-      </c>
-      <c r="U34" t="inlineStr">
-        <is>
-          <t>Mal manejo</t>
-        </is>
-      </c>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>BRINKS</t>
-        </is>
-      </c>
-      <c r="W34" t="inlineStr">
-        <is>
-          <t>FUNCIONARIOS</t>
-        </is>
-      </c>
-      <c r="X34">
-        <f>EXACT(TRIM(UPPER(V34)), TRIM(UPPER(W34)))</f>
-        <v/>
-      </c>
-      <c r="Y34" t="inlineStr"/>
-      <c r="Z34" t="n">
-        <v>1</v>
-      </c>
-      <c r="AA34" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB34" s="1" t="n">
-        <v>46214.46508101852</v>
-      </c>
-      <c r="AC34" s="1" t="n">
-        <v>46214.4650925926</v>
-      </c>
-      <c r="AD34" s="1" t="n">
-        <v>46214.47326388889</v>
-      </c>
-      <c r="AE34" t="n">
-        <v>707</v>
-      </c>
-      <c r="AF34" t="inlineStr">
-        <is>
-          <t>[2026-07-11 11:13:19] Jhon Fredy Ocampo Yepez: Mal manejo por no desarme de particion</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>FAA6FA10-0FB6-47F7-8B2B-80AC373C2FA3</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>D0705EFA-4C24-4253-84E9-FE31929F07DB</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>7482</v>
-      </c>
-      <c r="D35" t="n">
-        <v>7121</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>ATM</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>BOG Y SABANA</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>CUNDINAMARCA</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>BOGOTÁ, D.C.</t>
-        </is>
-      </c>
-      <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="n">
-        <v>1</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>WF 1047 - ZO01-Zonas 24H-ATM-AP:Disarm</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>activación perimetral</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>activación perimetral atm</t>
-        </is>
-      </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>7121 C MULTIFUNCIONAL PLAZA CLARO - 7482 - ATL - DIEBOLD</t>
-        </is>
-      </c>
-      <c r="P35" t="inlineStr">
-        <is>
-          <t>Honeywell7810PC-7482-54-2</t>
-        </is>
-      </c>
-      <c r="Q35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MAGNETICO CONTRATAPA INFERIOR CAJERO </t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Honeywell</t>
-        </is>
-      </c>
-      <c r="S35" t="n">
-        <v>0</v>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>JHON DAIRO ESCOBAR GARCIA</t>
-        </is>
-      </c>
-      <c r="U35" t="inlineStr">
-        <is>
-          <t>Falso positivo</t>
-        </is>
-      </c>
-      <c r="V35" t="inlineStr"/>
-      <c r="W35" t="inlineStr">
-        <is>
-          <t>ATLAS</t>
-        </is>
-      </c>
-      <c r="X35">
-        <f>EXACT(TRIM(UPPER(V35)), TRIM(UPPER(W35)))</f>
-        <v/>
-      </c>
-      <c r="Y35" t="inlineStr"/>
-      <c r="Z35" t="n">
-        <v>4</v>
-      </c>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>Oportuno</t>
-        </is>
-      </c>
-      <c r="AB35" s="1" t="n">
-        <v>46216.26837962963</v>
-      </c>
-      <c r="AC35" s="1" t="n">
-        <v>46216.26842592593</v>
-      </c>
-      <c r="AD35" s="1" t="n">
-        <v>46216.47231481481</v>
-      </c>
-      <c r="AE35" t="n">
-        <v>17620</v>
-      </c>
-      <c r="AF35" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>